<commit_message>
T-2792, T-2799, T-2980: Preserve wagon charts and complete transport references
</commit_message>
<xml_diff>
--- a/chicago/reference/resident-research/T-0462/T-0462_resident_research_working.xlsx
+++ b/chicago/reference/resident-research/T-0462/T-0462_resident_research_working.xlsx
@@ -9270,7 +9270,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>nwchicago_elijah_wentworth: https://nwchicagohistory.org/wp-content/uploads/2020/09/NWCHSJan-2020.pdf — named person or event entry | kinzie_waubun_1856: https://www.authorama.com/wau-bun-19.html — ch. XVII, 'Chicago in 1831'</t>
+          <t>nwchicago_elijah_wentworth: https://nwchicagohistory.org/wp-content/uploads/2020/09/NWCHSJan-2020.pdf — named person or event entry | kinzie_waubun_1856: https://www.authorama.com/wau-bun-19.html — ch. XVII, 'Chicago in 1831'; first 1856 edition printed pp. 210/221 (1812 baggage wagons); ch. XXIII 'Second Sight—Hickory Creek', p. 297 (1831 light dearborn wagon), and ch. XXIV 'Return to Fort Winnebago', p. 302 (pair of travelling horses), IA waubunearlydayin00kinz_0 scans 0309/0314</t>
         </is>
       </c>
       <c r="AC71" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="AF71" t="inlineStr">
         <is>
-          <t>nwchicago_elijah_wentworth: Reviewed for T-0462. Used only to the degree described in the resident research review; identity candidates remain unasserted. | kinzie_waubun_1856: The only near-contemporary descriptive text for the Wolf Point buildings. Load-bearing for the Sauganash: 'a pretentious white two-story building, with bright-blue wooden shutters, the admiration of all the little circle at Wolf Point.' Written 25 years after the events and describing 1831, not 1835 — hence tier 2 and the describes_date field. Also the source for the Indian Agency house ('logs hewed and squared, with a centre, two wings') and for the Wolf Point name deriving from an Indian resident called Moa-way, 'the Wolf'.</t>
+          <t>nwchicago_elijah_wentworth: Reviewed for T-0462. Used only to the degree described in the resident research review; identity candidates remain unasserted. | kinzie_waubun_1856: The only near-contemporary descriptive text for the Wolf Point buildings. Load-bearing for the Sauganash: 'a pretentious white two-story building, with bright-blue wooden shutters, the admiration of all the little circle at Wolf Point.' Written 25 years after the events and describing 1831, not 1835 — hence tier 2 and the describes_date field. Also the source for the Indian Agency house ('logs hewed and squared, with a centre, two wings') and for the Wolf Point name deriving from an Indian resident called Moa-way, 'the Wolf'. Vehicle use: p297 names Kercheval bringing a light dearborn wagon from Detroit, purchased by John Harris Kinzie for his mother and nephew; p302 names a pair of travelling horses. This is the1831 journey, not1812 and not proof the same wagon stood in Chicago1835. Maker, measurements, roof/curtains, paint and exact1835 placement are not supplied.</t>
         </is>
       </c>
       <c r="AG71" t="inlineStr">
@@ -11839,12 +11839,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ch. XVII, 'Chicago in 1831'</t>
+          <t>ch. XVII, 'Chicago in 1831'; first 1856 edition printed pp. 210/221 (1812 baggage wagons); ch. XXIII 'Second Sight—Hickory Creek', p. 297 (1831 light dearborn wagon), and ch. XXIV 'Return to Fort Winnebago', p. 302 (pair of travelling horses), IA waubunearlydayin00kinz_0 scans 0309/0314</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>The only near-contemporary descriptive text for the Wolf Point buildings. Load-bearing for the Sauganash: 'a pretentious white two-story building, with bright-blue wooden shutters, the admiration of all the little circle at Wolf Point.' Written 25 years after the events and describing 1831, not 1835 — hence tier 2 and the describes_date field. Also the source for the Indian Agency house ('logs hewed and squared, with a centre, two wings') and for the Wolf Point name deriving from an Indian resident called Moa-way, 'the Wolf'.</t>
+          <t>The only near-contemporary descriptive text for the Wolf Point buildings. Load-bearing for the Sauganash: 'a pretentious white two-story building, with bright-blue wooden shutters, the admiration of all the little circle at Wolf Point.' Written 25 years after the events and describing 1831, not 1835 — hence tier 2 and the describes_date field. Also the source for the Indian Agency house ('logs hewed and squared, with a centre, two wings') and for the Wolf Point name deriving from an Indian resident called Moa-way, 'the Wolf'. Vehicle use: p297 names Kercheval bringing a light dearborn wagon from Detroit, purchased by John Harris Kinzie for his mother and nephew; p302 names a pair of travelling horses. This is the1831 journey, not1812 and not proof the same wagon stood in Chicago1835. Maker, measurements, roof/curtains, paint and exact1835 placement are not supplied.</t>
         </is>
       </c>
     </row>

</xml_diff>